<commit_message>
Widen process flow, 30-day two-refiner Gantt, ARS from July 2027
- Slides 1-2: remove right-side condition panels and stretch the process
  flow across the slide (icons keep aspect ratio, connectors re-snapped)
- Slide 2: two-refiner staggered Gantt now spans day 1-30 (720 h) with
  inspection, 5 Gal filling and cumulative output rows
- ARS operation start set to 2027-07 for both EZChem and Hansol in the
  schedule table, slide text and workbook input

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BC5y8SeUSwKmhRPtP1c7Lt
</commit_message>
<xml_diff>
--- a/SKTC_CpZr_Capacity_RawData_Calculation_2026_2028.xlsx
+++ b/SKTC_CpZr_Capacity_RawData_Calculation_2026_2028.xlsx
@@ -3780,7 +3780,64 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">2028</t>
+      <t xml:space="preserve">ARS </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">운영 시점 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2027</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">년 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">7</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">월 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">· 2028</t>
     </r>
     <r>
       <rPr>
@@ -3843,142 +3900,45 @@
         <rFont val="Noto Sans CJK SC"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">첨부 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">PPT 2</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">장 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">'ARS 200 L </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">운영 계획 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">('26 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">설치 → </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">'27~)'</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">근거는 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">'27~ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">운영 계획뿐 — 전환 월 미확정</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">확인 필요 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">한솔 </t>
+      <t xml:space="preserve">사용자 지시 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(ARS </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">운영 시점 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2027</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">년 </t>
     </r>
     <r>
       <rPr>
@@ -3997,7 +3957,7 @@
         <rFont val="Noto Sans CJK SC"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">월 전환 자동 적용 안 함</t>
+      <t xml:space="preserve">월</t>
     </r>
     <r>
       <rPr>
@@ -4008,6 +3968,55 @@
         <charset val="1"/>
       </rPr>
       <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">이지켐</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">한솔 동일 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">'27.7~ ARS · '27.1~6 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">수동</t>
     </r>
   </si>
   <si>
@@ -21297,17 +21306,133 @@
         <rFont val="Noto Sans CJK SC"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">이지켐 수동 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">· </t>
+      <t xml:space="preserve">이지켐</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">한솔 수동 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(~'27.6)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">현재 조건 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(03 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">선택 간격</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">공사</t>
+  </si>
+  <si>
+    <t xml:space="preserve">가동 여부 미확인</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1·2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">개선 적용 생산</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">대</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">시간차 병행</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">이지켐</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
     </r>
     <r>
       <rPr>
@@ -21326,151 +21451,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">'27.1~6 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">수동</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">현재 조건 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(03 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">선택 간격</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">공사</t>
-  </si>
-  <si>
-    <t xml:space="preserve">가동 여부 미확인</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1·2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">개선 적용 생산</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">2</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">대</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">시간차 병행</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">한솔 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">ARS · </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">이지켐 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">ARS(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">전환 월 확인</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
+      <t xml:space="preserve">ARS ('27.7~)</t>
     </r>
   </si>
   <si>
@@ -26621,17 +26602,55 @@
         <rFont val="Noto Sans CJK SC"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">한솔 수동</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">·ARS </t>
+      <t xml:space="preserve">한솔 수동 충진시간 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">· </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">이지켐</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">한솔 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">ARS </t>
     </r>
     <r>
       <rPr>
@@ -26650,54 +26669,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">· </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">이지켐 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">ARS </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">전환 월</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">·</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">시간</t>
+      <t xml:space="preserve">('27.7~)</t>
     </r>
   </si>
   <si>
@@ -28208,11 +28180,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="96233383"/>
-        <c:axId val="20192760"/>
+        <c:axId val="39492676"/>
+        <c:axId val="19255739"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="96233383"/>
+        <c:axId val="39492676"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -28244,7 +28216,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="20192760"/>
+        <c:crossAx val="19255739"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -28252,7 +28224,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="20192760"/>
+        <c:axId val="19255739"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -28294,7 +28266,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="96233383"/>
+        <c:crossAx val="39492676"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -28939,11 +28911,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="83994883"/>
-        <c:axId val="32617448"/>
+        <c:axId val="38867338"/>
+        <c:axId val="50331020"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="83994883"/>
+        <c:axId val="38867338"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -28975,7 +28947,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="32617448"/>
+        <c:crossAx val="50331020"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -28983,7 +28955,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="32617448"/>
+        <c:axId val="50331020"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -29025,7 +28997,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="83994883"/>
+        <c:crossAx val="38867338"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -30272,12 +30244,12 @@
         <v>140</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="13" t="s">
         <v>141</v>
       </c>
       <c r="B47" s="21" t="n">
-        <v>46388</v>
+        <v>46569</v>
       </c>
       <c r="C47" s="13" t="s">
         <v>134</v>
@@ -46804,15 +46776,15 @@
       </c>
       <c r="AF18" s="13" t="str">
         <f aca="false">IF(AD18=0,"-",IF(A18&gt;=01_Inputs!$B$47,"ARS","수동"))</f>
-        <v>ARS</v>
+        <v>수동</v>
       </c>
       <c r="AG18" s="13" t="str">
         <f aca="false">IF(AE18=0,"-",IF(A18&gt;=01_Inputs!$B$46,"ARS","수동"))</f>
         <v>수동</v>
       </c>
-      <c r="AH18" s="15" t="str">
+      <c r="AH18" s="15" t="n">
         <f aca="false">IF(AD18=0,0,IF(AF18="수동",AD18*01_Inputs!$B$34,IF(ISNUMBER(01_Inputs!$B$36),AD18*01_Inputs!$B$36,"미확인")))</f>
-        <v>미확인</v>
+        <v>32</v>
       </c>
       <c r="AI18" s="15" t="str">
         <f aca="false">IF(AE18=0,0,IF(AG18="수동",IF(ISNUMBER(01_Inputs!$B$35),AE18*01_Inputs!$B$35,"미확인"),IF(ISNUMBER(01_Inputs!$B$37),AE18*01_Inputs!$B$37,"미확인")))</f>
@@ -46820,7 +46792,7 @@
       </c>
       <c r="AJ18" s="15" t="str">
         <f aca="false">IF(AND(ISNUMBER(AH18),ISNUMBER(AI18)),AH18+AI18,"부분 "&amp;TEXT(N(AH18)+N(AI18),"0")&amp;" h + 미확인")</f>
-        <v>부분 0 h + 미확인</v>
+        <v>부분 32 h + 미확인</v>
       </c>
       <c r="AK18" s="15" t="n">
         <f aca="false">(AD18+AE18)*01_Inputs!$B$38</f>
@@ -47027,15 +46999,15 @@
       </c>
       <c r="AF19" s="13" t="str">
         <f aca="false">IF(AD19=0,"-",IF(A19&gt;=01_Inputs!$B$47,"ARS","수동"))</f>
-        <v>ARS</v>
+        <v>수동</v>
       </c>
       <c r="AG19" s="13" t="str">
         <f aca="false">IF(AE19=0,"-",IF(A19&gt;=01_Inputs!$B$46,"ARS","수동"))</f>
         <v>수동</v>
       </c>
-      <c r="AH19" s="15" t="str">
+      <c r="AH19" s="15" t="n">
         <f aca="false">IF(AD19=0,0,IF(AF19="수동",AD19*01_Inputs!$B$34,IF(ISNUMBER(01_Inputs!$B$36),AD19*01_Inputs!$B$36,"미확인")))</f>
-        <v>미확인</v>
+        <v>32</v>
       </c>
       <c r="AI19" s="15" t="str">
         <f aca="false">IF(AE19=0,0,IF(AG19="수동",IF(ISNUMBER(01_Inputs!$B$35),AE19*01_Inputs!$B$35,"미확인"),IF(ISNUMBER(01_Inputs!$B$37),AE19*01_Inputs!$B$37,"미확인")))</f>
@@ -47043,7 +47015,7 @@
       </c>
       <c r="AJ19" s="15" t="str">
         <f aca="false">IF(AND(ISNUMBER(AH19),ISNUMBER(AI19)),AH19+AI19,"부분 "&amp;TEXT(N(AH19)+N(AI19),"0")&amp;" h + 미확인")</f>
-        <v>부분 0 h + 미확인</v>
+        <v>부분 32 h + 미확인</v>
       </c>
       <c r="AK19" s="15" t="n">
         <f aca="false">(AD19+AE19)*01_Inputs!$B$38</f>
@@ -47250,15 +47222,15 @@
       </c>
       <c r="AF20" s="13" t="str">
         <f aca="false">IF(AD20=0,"-",IF(A20&gt;=01_Inputs!$B$47,"ARS","수동"))</f>
-        <v>ARS</v>
+        <v>수동</v>
       </c>
       <c r="AG20" s="13" t="str">
         <f aca="false">IF(AE20=0,"-",IF(A20&gt;=01_Inputs!$B$46,"ARS","수동"))</f>
         <v>수동</v>
       </c>
-      <c r="AH20" s="15" t="str">
+      <c r="AH20" s="15" t="n">
         <f aca="false">IF(AD20=0,0,IF(AF20="수동",AD20*01_Inputs!$B$34,IF(ISNUMBER(01_Inputs!$B$36),AD20*01_Inputs!$B$36,"미확인")))</f>
-        <v>미확인</v>
+        <v>32</v>
       </c>
       <c r="AI20" s="15" t="str">
         <f aca="false">IF(AE20=0,0,IF(AG20="수동",IF(ISNUMBER(01_Inputs!$B$35),AE20*01_Inputs!$B$35,"미확인"),IF(ISNUMBER(01_Inputs!$B$37),AE20*01_Inputs!$B$37,"미확인")))</f>
@@ -47266,7 +47238,7 @@
       </c>
       <c r="AJ20" s="15" t="str">
         <f aca="false">IF(AND(ISNUMBER(AH20),ISNUMBER(AI20)),AH20+AI20,"부분 "&amp;TEXT(N(AH20)+N(AI20),"0")&amp;" h + 미확인")</f>
-        <v>부분 0 h + 미확인</v>
+        <v>부분 32 h + 미확인</v>
       </c>
       <c r="AK20" s="15" t="n">
         <f aca="false">(AD20+AE20)*01_Inputs!$B$38</f>
@@ -47473,15 +47445,15 @@
       </c>
       <c r="AF21" s="13" t="str">
         <f aca="false">IF(AD21=0,"-",IF(A21&gt;=01_Inputs!$B$47,"ARS","수동"))</f>
-        <v>ARS</v>
+        <v>수동</v>
       </c>
       <c r="AG21" s="13" t="str">
         <f aca="false">IF(AE21=0,"-",IF(A21&gt;=01_Inputs!$B$46,"ARS","수동"))</f>
         <v>수동</v>
       </c>
-      <c r="AH21" s="15" t="str">
+      <c r="AH21" s="15" t="n">
         <f aca="false">IF(AD21=0,0,IF(AF21="수동",AD21*01_Inputs!$B$34,IF(ISNUMBER(01_Inputs!$B$36),AD21*01_Inputs!$B$36,"미확인")))</f>
-        <v>미확인</v>
+        <v>32</v>
       </c>
       <c r="AI21" s="15" t="str">
         <f aca="false">IF(AE21=0,0,IF(AG21="수동",IF(ISNUMBER(01_Inputs!$B$35),AE21*01_Inputs!$B$35,"미확인"),IF(ISNUMBER(01_Inputs!$B$37),AE21*01_Inputs!$B$37,"미확인")))</f>
@@ -47489,7 +47461,7 @@
       </c>
       <c r="AJ21" s="15" t="str">
         <f aca="false">IF(AND(ISNUMBER(AH21),ISNUMBER(AI21)),AH21+AI21,"부분 "&amp;TEXT(N(AH21)+N(AI21),"0")&amp;" h + 미확인")</f>
-        <v>부분 0 h + 미확인</v>
+        <v>부분 32 h + 미확인</v>
       </c>
       <c r="AK21" s="15" t="n">
         <f aca="false">(AD21+AE21)*01_Inputs!$B$38</f>
@@ -47696,15 +47668,15 @@
       </c>
       <c r="AF22" s="13" t="str">
         <f aca="false">IF(AD22=0,"-",IF(A22&gt;=01_Inputs!$B$47,"ARS","수동"))</f>
-        <v>ARS</v>
+        <v>수동</v>
       </c>
       <c r="AG22" s="13" t="str">
         <f aca="false">IF(AE22=0,"-",IF(A22&gt;=01_Inputs!$B$46,"ARS","수동"))</f>
         <v>수동</v>
       </c>
-      <c r="AH22" s="15" t="str">
+      <c r="AH22" s="15" t="n">
         <f aca="false">IF(AD22=0,0,IF(AF22="수동",AD22*01_Inputs!$B$34,IF(ISNUMBER(01_Inputs!$B$36),AD22*01_Inputs!$B$36,"미확인")))</f>
-        <v>미확인</v>
+        <v>32</v>
       </c>
       <c r="AI22" s="15" t="str">
         <f aca="false">IF(AE22=0,0,IF(AG22="수동",IF(ISNUMBER(01_Inputs!$B$35),AE22*01_Inputs!$B$35,"미확인"),IF(ISNUMBER(01_Inputs!$B$37),AE22*01_Inputs!$B$37,"미확인")))</f>
@@ -47712,7 +47684,7 @@
       </c>
       <c r="AJ22" s="15" t="str">
         <f aca="false">IF(AND(ISNUMBER(AH22),ISNUMBER(AI22)),AH22+AI22,"부분 "&amp;TEXT(N(AH22)+N(AI22),"0")&amp;" h + 미확인")</f>
-        <v>부분 0 h + 미확인</v>
+        <v>부분 32 h + 미확인</v>
       </c>
       <c r="AK22" s="15" t="n">
         <f aca="false">(AD22+AE22)*01_Inputs!$B$38</f>
@@ -47919,15 +47891,15 @@
       </c>
       <c r="AF23" s="13" t="str">
         <f aca="false">IF(AD23=0,"-",IF(A23&gt;=01_Inputs!$B$47,"ARS","수동"))</f>
-        <v>ARS</v>
+        <v>수동</v>
       </c>
       <c r="AG23" s="13" t="str">
         <f aca="false">IF(AE23=0,"-",IF(A23&gt;=01_Inputs!$B$46,"ARS","수동"))</f>
         <v>수동</v>
       </c>
-      <c r="AH23" s="15" t="str">
+      <c r="AH23" s="15" t="n">
         <f aca="false">IF(AD23=0,0,IF(AF23="수동",AD23*01_Inputs!$B$34,IF(ISNUMBER(01_Inputs!$B$36),AD23*01_Inputs!$B$36,"미확인")))</f>
-        <v>미확인</v>
+        <v>32</v>
       </c>
       <c r="AI23" s="15" t="str">
         <f aca="false">IF(AE23=0,0,IF(AG23="수동",IF(ISNUMBER(01_Inputs!$B$35),AE23*01_Inputs!$B$35,"미확인"),IF(ISNUMBER(01_Inputs!$B$37),AE23*01_Inputs!$B$37,"미확인")))</f>
@@ -47935,7 +47907,7 @@
       </c>
       <c r="AJ23" s="15" t="str">
         <f aca="false">IF(AND(ISNUMBER(AH23),ISNUMBER(AI23)),AH23+AI23,"부분 "&amp;TEXT(N(AH23)+N(AI23),"0")&amp;" h + 미확인")</f>
-        <v>부분 0 h + 미확인</v>
+        <v>부분 32 h + 미확인</v>
       </c>
       <c r="AK23" s="15" t="n">
         <f aca="false">(AD23+AE23)*01_Inputs!$B$38</f>
@@ -52203,7 +52175,7 @@
       </c>
       <c r="AH43" s="53" t="str">
         <f aca="false">IF(COUNTIF(AH18:AH29,"미확인")&gt;0,"부분 "&amp;TEXT(SUM(AH18:AH29),"0")&amp;" h + 미확인",SUM(AH18:AH29))</f>
-        <v>부분 0 h + 미확인</v>
+        <v>부분 192 h + 미확인</v>
       </c>
       <c r="AI43" s="53" t="str">
         <f aca="false">IF(COUNTIF(AI18:AI29,"미확인")&gt;0,"부분 "&amp;TEXT(SUM(AI18:AI29),"0")&amp;" h + 미확인",SUM(AI18:AI29))</f>
@@ -52684,7 +52656,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="24.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
         <v>762</v>
       </c>
@@ -56137,7 +56109,7 @@
       </c>
       <c r="B88" s="50" t="str">
         <f aca="false">04_Monthly_2026_2028!$AH$43</f>
-        <v>부분 0 h + 미확인</v>
+        <v>부분 192 h + 미확인</v>
       </c>
       <c r="C88" s="9" t="s">
         <v>42</v>

</xml_diff>

<commit_message>
Reflect day-shift-only filling (08-17, lunch excluded = 8 h/day)
- Excel: shift start/end/lunch inputs drive WH_DAY; labels use 상근조 instead of 1교대
- PPT: slides 1, 3, 11, 13 describe 5 Gal 18 h as ~2 days on the day shift
- Prompt: data, slide specs, Excel row addresses and checks updated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BC5y8SeUSwKmhRPtP1c7Lt
</commit_message>
<xml_diff>
--- a/SKTC_CpZr_Capacity_RawData_Calculation_2026_2028.xlsx
+++ b/SKTC_CpZr_Capacity_RawData_Calculation_2026_2028.xlsx
@@ -49,21 +49,24 @@
     <definedName name="ARS_HS_S">'01_입력'!$C$40</definedName>
     <definedName name="ARS_EZ_T">'01_입력'!$C$41</definedName>
     <definedName name="ARS_HS_T">'01_입력'!$C$42</definedName>
-    <definedName name="WH_DAY">'01_입력'!$C$43</definedName>
-    <definedName name="WD_MON">'01_입력'!$C$44</definedName>
-    <definedName name="FILL_5G_EL">'01_입력'!$C$45</definedName>
-    <definedName name="B_SIZE">'01_입력'!$C$59</definedName>
-    <definedName name="B_YIELD">'01_입력'!$C$60</definedName>
-    <definedName name="KG_B">'01_입력'!$C$61</definedName>
-    <definedName name="B_TIME">'01_입력'!$C$62</definedName>
-    <definedName name="UNIT_RM">'01_입력'!$C$63</definedName>
-    <definedName name="MB_ONE">'01_입력'!$C$64</definedName>
-    <definedName name="MB_TWO">'01_입력'!$C$65</definedName>
-    <definedName name="MB_MAINT">'01_입력'!$C$66</definedName>
-    <definedName name="CAPA_NOW">'01_입력'!$C$70</definedName>
-    <definedName name="CAPA_ADD">'01_입력'!$C$71</definedName>
-    <definedName name="CAPA_RF">'01_입력'!$C$72</definedName>
-    <definedName name="CAPA_TWO">'01_입력'!$C$73</definedName>
+    <definedName name="SH_START">'01_입력'!$C$43</definedName>
+    <definedName name="SH_END">'01_입력'!$C$44</definedName>
+    <definedName name="SH_LUNCH">'01_입력'!$C$45</definedName>
+    <definedName name="WH_DAY">'01_입력'!$C$46</definedName>
+    <definedName name="WD_MON">'01_입력'!$C$47</definedName>
+    <definedName name="FILL_5G_EL">'01_입력'!$C$48</definedName>
+    <definedName name="B_SIZE">'01_입력'!$C$62</definedName>
+    <definedName name="B_YIELD">'01_입력'!$C$63</definedName>
+    <definedName name="KG_B">'01_입력'!$C$64</definedName>
+    <definedName name="B_TIME">'01_입력'!$C$65</definedName>
+    <definedName name="UNIT_RM">'01_입력'!$C$66</definedName>
+    <definedName name="MB_ONE">'01_입력'!$C$67</definedName>
+    <definedName name="MB_TWO">'01_입력'!$C$68</definedName>
+    <definedName name="MB_MAINT">'01_입력'!$C$69</definedName>
+    <definedName name="CAPA_NOW">'01_입력'!$C$73</definedName>
+    <definedName name="CAPA_ADD">'01_입력'!$C$74</definedName>
+    <definedName name="CAPA_RF">'01_입력'!$C$75</definedName>
+    <definedName name="CAPA_TWO">'01_입력'!$C$76</definedName>
     <definedName name="PL_B">'03_Batch주기'!$C$19</definedName>
     <definedName name="PL_KG">'03_Batch주기'!$C$20</definedName>
     <definedName name="CYC_ASIS">'03_Batch주기'!$C$21</definedName>
@@ -783,7 +786,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:M89"/>
+  <dimension ref="B1:M92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -1396,7 +1399,7 @@
         </is>
       </c>
       <c r="C41" s="17">
-        <f>IF(COUNT(C48:C53)=0,"",SUM(C48:C53))</f>
+        <f>IF(COUNT(C51:C56)=0,"",SUM(C51:C56))</f>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
@@ -1416,7 +1419,7 @@
         </is>
       </c>
       <c r="C42" s="17">
-        <f>IF(COUNT(D48:D53)=0,"",SUM(D48:D53))</f>
+        <f>IF(COUNT(D51:D56)=0,"",SUM(D51:D56))</f>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
@@ -1432,35 +1435,35 @@
     <row r="43">
       <c r="B43" s="10" t="inlineStr">
         <is>
-          <t>글로브 박스 근무시간</t>
-        </is>
-      </c>
-      <c r="C43" s="11" t="n">
+          <t>충진 근무 시작 (상근조)</t>
+        </is>
+      </c>
+      <c r="C43" s="14" t="n">
         <v>8</v>
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>h/일</t>
+          <t>시</t>
         </is>
       </c>
       <c r="E43" s="12" t="inlineStr">
         <is>
-          <t>1교대 기준</t>
+          <t>충진은 보통 상근조만 진행</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>월 근무일</t>
+          <t>충진 근무 종료 (상근조)</t>
         </is>
       </c>
       <c r="C44" s="14" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>일/월</t>
+          <t>시</t>
         </is>
       </c>
       <c r="E44" s="12" t="inlineStr"/>
@@ -1468,11 +1471,11 @@
     <row r="45">
       <c r="B45" s="10" t="inlineStr">
         <is>
-          <t>5 Gal 9병 충진 경과 (근무시간 반영)</t>
+          <t>점심시간 (12:00~13:00)</t>
         </is>
       </c>
       <c r="C45" s="11" t="n">
-        <v>48</v>
+        <v>1</v>
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
@@ -1481,66 +1484,93 @@
       </c>
       <c r="E45" s="12" t="inlineStr">
         <is>
-          <t>현장 설명 약 2일 (작업 18 h)</t>
+          <t>근무시간에서 제외</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" s="10" t="inlineStr">
+        <is>
+          <t>충진 근무시간 (상근조)</t>
+        </is>
+      </c>
+      <c r="C46" s="17">
+        <f>SH_END-SH_START-SH_LUNCH</f>
+        <v>8</v>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>h/일</t>
+        </is>
+      </c>
+      <c r="E46" s="12" t="inlineStr">
+        <is>
+          <t>08:00~17:00 − 점심 1 h = 8 h/일</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="B47" s="8" t="inlineStr">
-        <is>
-          <t>ARS 작업 단계 (h/용기)</t>
-        </is>
-      </c>
-      <c r="C47" s="9" t="inlineStr">
-        <is>
-          <t>이지켐</t>
-        </is>
-      </c>
-      <c r="D47" s="9" t="inlineStr">
-        <is>
-          <t>한솔</t>
-        </is>
-      </c>
-      <c r="E47" s="8" t="inlineStr">
-        <is>
-          <t>수동과 ARS의 전체 시간 차이 확인용</t>
-        </is>
-      </c>
+      <c r="B47" s="10" t="inlineStr">
+        <is>
+          <t>월 근무일</t>
+        </is>
+      </c>
+      <c r="C47" s="14" t="n">
+        <v>22</v>
+      </c>
+      <c r="D47" s="5" t="inlineStr">
+        <is>
+          <t>일/월</t>
+        </is>
+      </c>
+      <c r="E47" s="12" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>용기 준비</t>
-        </is>
-      </c>
-      <c r="C48" s="16" t="n"/>
-      <c r="D48" s="16" t="n"/>
-      <c r="E48" s="18" t="inlineStr"/>
-    </row>
-    <row r="49">
-      <c r="B49" s="10" t="inlineStr">
-        <is>
-          <t>투입·반출</t>
-        </is>
-      </c>
-      <c r="C49" s="16" t="n"/>
-      <c r="D49" s="16" t="n"/>
-      <c r="E49" s="18" t="inlineStr"/>
+          <t>5 Gal 9병 충진 경과 (상근조 기준)</t>
+        </is>
+      </c>
+      <c r="C48" s="11" t="n">
+        <v>48</v>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E48" s="12" t="inlineStr">
+        <is>
+          <t>18 h ÷ 상근조 8 h/일 = 2.25 근무일 → 현장 설명 약 2일 (48 h)</t>
+        </is>
+      </c>
     </row>
     <row r="50">
-      <c r="B50" s="10" t="inlineStr">
-        <is>
-          <t>퍼지</t>
-        </is>
-      </c>
-      <c r="C50" s="16" t="n"/>
-      <c r="D50" s="16" t="n"/>
-      <c r="E50" s="18" t="inlineStr"/>
+      <c r="B50" s="8" t="inlineStr">
+        <is>
+          <t>ARS 작업 단계 (h/용기)</t>
+        </is>
+      </c>
+      <c r="C50" s="9" t="inlineStr">
+        <is>
+          <t>이지켐</t>
+        </is>
+      </c>
+      <c r="D50" s="9" t="inlineStr">
+        <is>
+          <t>한솔</t>
+        </is>
+      </c>
+      <c r="E50" s="8" t="inlineStr">
+        <is>
+          <t>수동과 ARS의 전체 시간 차이 확인용</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="B51" s="10" t="inlineStr">
         <is>
-          <t>실제 충진</t>
+          <t>용기 준비</t>
         </is>
       </c>
       <c r="C51" s="16" t="n"/>
@@ -1550,7 +1580,7 @@
     <row r="52">
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>설비 전환</t>
+          <t>투입·반출</t>
         </is>
       </c>
       <c r="C52" s="16" t="n"/>
@@ -1560,7 +1590,7 @@
     <row r="53">
       <c r="B53" s="10" t="inlineStr">
         <is>
-          <t>검사·OQC</t>
+          <t>퍼지</t>
         </is>
       </c>
       <c r="C53" s="16" t="n"/>
@@ -1570,7 +1600,7 @@
     <row r="54">
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t>작업자 투입시간</t>
+          <t>실제 충진</t>
         </is>
       </c>
       <c r="C54" s="16" t="n"/>
@@ -1580,456 +1610,486 @@
     <row r="55">
       <c r="B55" s="10" t="inlineStr">
         <is>
-          <t>설비 점유시간</t>
+          <t>설비 전환</t>
         </is>
       </c>
       <c r="C55" s="16" t="n"/>
       <c r="D55" s="16" t="n"/>
       <c r="E55" s="18" t="inlineStr"/>
     </row>
-    <row r="57" ht="20" customHeight="1">
-      <c r="B57" s="7" t="inlineStr">
+    <row r="56">
+      <c r="B56" s="10" t="inlineStr">
+        <is>
+          <t>검사·OQC</t>
+        </is>
+      </c>
+      <c r="C56" s="16" t="n"/>
+      <c r="D56" s="16" t="n"/>
+      <c r="E56" s="18" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="B57" s="10" t="inlineStr">
+        <is>
+          <t>작업자 투입시간</t>
+        </is>
+      </c>
+      <c r="C57" s="16" t="n"/>
+      <c r="D57" s="16" t="n"/>
+      <c r="E57" s="18" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="B58" s="10" t="inlineStr">
+        <is>
+          <t>설비 점유시간</t>
+        </is>
+      </c>
+      <c r="C58" s="16" t="n"/>
+      <c r="D58" s="16" t="n"/>
+      <c r="E58" s="18" t="inlineStr"/>
+    </row>
+    <row r="60" ht="20" customHeight="1">
+      <c r="B60" s="7" t="inlineStr">
         <is>
           <t>D. Batch 생산량 (생산팀 협의)</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="B58" s="8" t="inlineStr">
+    <row r="61">
+      <c r="B61" s="8" t="inlineStr">
         <is>
           <t>항목</t>
         </is>
       </c>
-      <c r="C58" s="9" t="inlineStr">
+      <c r="C61" s="9" t="inlineStr">
         <is>
           <t>값</t>
         </is>
       </c>
-      <c r="D58" s="9" t="inlineStr">
+      <c r="D61" s="9" t="inlineStr">
         <is>
           <t>단위</t>
         </is>
       </c>
-      <c r="E58" s="8" t="inlineStr">
+      <c r="E61" s="8" t="inlineStr">
         <is>
           <t>설명</t>
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="B59" s="10" t="inlineStr">
+    <row r="62">
+      <c r="B62" s="10" t="inlineStr">
         <is>
           <t>Batch size</t>
         </is>
       </c>
-      <c r="C59" s="14" t="n">
+      <c r="C62" s="14" t="n">
         <v>200</v>
       </c>
-      <c r="D59" s="5" t="inlineStr">
+      <c r="D62" s="5" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="E59" s="12" t="inlineStr">
+      <c r="E62" s="12" t="inlineStr">
         <is>
           <t>생산팀 협의</t>
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="B60" s="10" t="inlineStr">
+    <row r="63">
+      <c r="B63" s="10" t="inlineStr">
         <is>
           <t>Yield</t>
         </is>
       </c>
-      <c r="C60" s="19" t="n">
+      <c r="C63" s="19" t="n">
         <v>0.99</v>
       </c>
-      <c r="D60" s="5" t="inlineStr">
+      <c r="D63" s="5" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E60" s="12" t="inlineStr"/>
-    </row>
-    <row r="61">
-      <c r="B61" s="10" t="inlineStr">
+      <c r="E63" s="12" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="B64" s="10" t="inlineStr">
         <is>
           <t>kg/Batch (Batch size × Yield)</t>
         </is>
       </c>
-      <c r="C61" s="20">
+      <c r="C64" s="20">
         <f>B_SIZE*B_YIELD</f>
         <v>198</v>
       </c>
-      <c r="D61" s="5" t="inlineStr">
+      <c r="D64" s="5" t="inlineStr">
         <is>
           <t>kg/Batch</t>
         </is>
       </c>
-      <c r="E61" s="12" t="inlineStr">
+      <c r="E64" s="12" t="inlineStr">
         <is>
           <t>200 × 99% = 198 kg</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="B62" s="10" t="inlineStr">
-        <is>
-          <t>Batch time (협의)</t>
-        </is>
-      </c>
-      <c r="C62" s="11" t="n">
-        <v>55</v>
-      </c>
-      <c r="D62" s="5" t="inlineStr">
-        <is>
-          <t>h</t>
-        </is>
-      </c>
-      <c r="E62" s="12" t="inlineStr">
-        <is>
-          <t>준비·투입 ~ FQC (IQC~FQC 57 h − IQC 2 h)</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="B63" s="10" t="inlineStr">
-        <is>
-          <t>원단위</t>
-        </is>
-      </c>
-      <c r="C63" s="21" t="n">
-        <v>1.01</v>
-      </c>
-      <c r="D63" s="5" t="inlineStr"/>
-      <c r="E63" s="12" t="inlineStr"/>
-    </row>
-    <row r="64">
-      <c r="B64" s="10" t="inlineStr">
-        <is>
-          <t>정제기 1대 월 Batch (계획)</t>
-        </is>
-      </c>
-      <c r="C64" s="14" t="n">
-        <v>12</v>
-      </c>
-      <c r="D64" s="5" t="inlineStr">
-        <is>
-          <t>Batch/월</t>
-        </is>
-      </c>
-      <c r="E64" s="12" t="inlineStr">
-        <is>
-          <t>12 × 198 = 2,376 kg</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="B65" s="10" t="inlineStr">
         <is>
-          <t>정제기 2대 월 Batch (계획)</t>
-        </is>
-      </c>
-      <c r="C65" s="14" t="n">
-        <v>20</v>
+          <t>Batch time (협의)</t>
+        </is>
+      </c>
+      <c r="C65" s="11" t="n">
+        <v>55</v>
       </c>
       <c r="D65" s="5" t="inlineStr">
         <is>
-          <t>Batch/월</t>
+          <t>h</t>
         </is>
       </c>
       <c r="E65" s="12" t="inlineStr">
         <is>
-          <t>20 × 198 = 3,960 kg</t>
+          <t>준비·투입 ~ FQC (IQC~FQC 57 h − IQC 2 h)</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="B66" s="10" t="inlineStr">
         <is>
+          <t>원단위</t>
+        </is>
+      </c>
+      <c r="C66" s="21" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="D66" s="5" t="inlineStr"/>
+      <c r="E66" s="12" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="B67" s="10" t="inlineStr">
+        <is>
+          <t>정제기 1대 월 Batch (계획)</t>
+        </is>
+      </c>
+      <c r="C67" s="14" t="n">
+        <v>12</v>
+      </c>
+      <c r="D67" s="5" t="inlineStr">
+        <is>
+          <t>Batch/월</t>
+        </is>
+      </c>
+      <c r="E67" s="12" t="inlineStr">
+        <is>
+          <t>12 × 198 = 2,376 kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="B68" s="10" t="inlineStr">
+        <is>
+          <t>정제기 2대 월 Batch (계획)</t>
+        </is>
+      </c>
+      <c r="C68" s="14" t="n">
+        <v>20</v>
+      </c>
+      <c r="D68" s="5" t="inlineStr">
+        <is>
+          <t>Batch/월</t>
+        </is>
+      </c>
+      <c r="E68" s="12" t="inlineStr">
+        <is>
+          <t>20 × 198 = 3,960 kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="B69" s="10" t="inlineStr">
+        <is>
           <t>대정비 월 Batch ('27.4)</t>
         </is>
       </c>
-      <c r="C66" s="14" t="n">
+      <c r="C69" s="14" t="n">
         <v>6</v>
       </c>
-      <c r="D66" s="5" t="inlineStr">
+      <c r="D69" s="5" t="inlineStr">
         <is>
           <t>Batch/월</t>
         </is>
       </c>
-      <c r="E66" s="12" t="inlineStr">
+      <c r="E69" s="12" t="inlineStr">
         <is>
           <t>6 × 198 = 1,188 kg</t>
         </is>
       </c>
     </row>
-    <row r="68" ht="20" customHeight="1">
-      <c r="B68" s="7" t="inlineStr">
+    <row r="71" ht="20" customHeight="1">
+      <c r="B71" s="7" t="inlineStr">
         <is>
           <t>E. Capa. 기준</t>
         </is>
       </c>
     </row>
-    <row r="69">
-      <c r="B69" s="8" t="inlineStr">
+    <row r="72">
+      <c r="B72" s="8" t="inlineStr">
         <is>
           <t>항목</t>
         </is>
       </c>
-      <c r="C69" s="9" t="inlineStr">
+      <c r="C72" s="9" t="inlineStr">
         <is>
           <t>값</t>
         </is>
       </c>
-      <c r="D69" s="9" t="inlineStr">
+      <c r="D72" s="9" t="inlineStr">
         <is>
           <t>단위</t>
         </is>
       </c>
-      <c r="E69" s="8" t="inlineStr">
+      <c r="E72" s="8" t="inlineStr">
         <is>
           <t>설명</t>
         </is>
       </c>
     </row>
-    <row r="70">
-      <c r="B70" s="10" t="inlineStr">
+    <row r="73">
+      <c r="B73" s="10" t="inlineStr">
         <is>
           <t>현재 연간 Capa.</t>
         </is>
       </c>
-      <c r="C70" s="22" t="n">
+      <c r="C73" s="22" t="n">
         <v>26.2</v>
       </c>
-      <c r="D70" s="5" t="inlineStr">
+      <c r="D73" s="5" t="inlineStr">
         <is>
           <t>t/년</t>
         </is>
       </c>
-      <c r="E70" s="12" t="inlineStr"/>
-    </row>
-    <row r="71">
-      <c r="B71" s="10" t="inlineStr">
+      <c r="E73" s="12" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="B74" s="10" t="inlineStr">
         <is>
           <t>리플럭스 증가분</t>
         </is>
       </c>
-      <c r="C71" s="22" t="n">
+      <c r="C74" s="22" t="n">
         <v>21</v>
       </c>
-      <c r="D71" s="5" t="inlineStr">
+      <c r="D74" s="5" t="inlineStr">
         <is>
           <t>t/년</t>
         </is>
       </c>
-      <c r="E71" s="12" t="inlineStr"/>
-    </row>
-    <row r="72">
-      <c r="B72" s="10" t="inlineStr">
+      <c r="E74" s="12" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="B75" s="10" t="inlineStr">
         <is>
           <t>개선 후 연간 Capa.</t>
         </is>
       </c>
-      <c r="C72" s="23">
+      <c r="C75" s="23">
         <f>CAPA_NOW+CAPA_ADD</f>
         <v>47.2</v>
       </c>
-      <c r="D72" s="5" t="inlineStr">
+      <c r="D75" s="5" t="inlineStr">
         <is>
           <t>t/년</t>
         </is>
       </c>
-      <c r="E72" s="12" t="inlineStr">
+      <c r="E75" s="12" t="inlineStr">
         <is>
           <t>현재의 2배(52.4) 아님 — Mix·Premix 준비 등</t>
         </is>
       </c>
     </row>
-    <row r="73">
-      <c r="B73" s="10" t="inlineStr">
+    <row r="76">
+      <c r="B76" s="10" t="inlineStr">
         <is>
           <t>정제기 2대 계획 연간 (20 Batch × 12)</t>
         </is>
       </c>
-      <c r="C73" s="23">
+      <c r="C76" s="23">
         <f>MB_TWO*KG_B*12/1000</f>
         <v>47.52</v>
       </c>
-      <c r="D73" s="5" t="inlineStr">
+      <c r="D76" s="5" t="inlineStr">
         <is>
           <t>t/년</t>
         </is>
       </c>
-      <c r="E73" s="12" t="inlineStr">
+      <c r="E76" s="12" t="inlineStr">
         <is>
           <t>47.2톤 계획 수준</t>
         </is>
       </c>
     </row>
-    <row r="75" ht="20" customHeight="1">
-      <c r="B75" s="7" t="inlineStr">
+    <row r="78" ht="20" customHeight="1">
+      <c r="B78" s="7" t="inlineStr">
         <is>
           <t>I. 생산계획 Batch 완료일 — 완료일 = 해당 Batch의 생산 및 충진 완료 예정일 (Batch마다 독립)</t>
         </is>
       </c>
     </row>
-    <row r="76">
-      <c r="B76" s="8" t="inlineStr">
+    <row r="79">
+      <c r="B79" s="8" t="inlineStr">
         <is>
           <t>Batch No.</t>
         </is>
       </c>
-      <c r="C76" s="9" t="inlineStr">
+      <c r="C79" s="9" t="inlineStr">
         <is>
           <t>완료일</t>
         </is>
       </c>
-      <c r="D76" s="8" t="inlineStr">
+      <c r="D79" s="8" t="inlineStr">
         <is>
           <t>비고</t>
         </is>
       </c>
-    </row>
-    <row r="77">
-      <c r="B77" s="24" t="inlineStr">
-        <is>
-          <t>#81</t>
-        </is>
-      </c>
-      <c r="C77" s="15" t="n">
-        <v>46293</v>
-      </c>
-      <c r="D77" s="18" t="inlineStr">
-        <is>
-          <t>9월 마지막 Batch (간격 기준점)</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="B78" s="24" t="inlineStr">
-        <is>
-          <t>#82</t>
-        </is>
-      </c>
-      <c r="C78" s="15" t="n">
-        <v>46296</v>
-      </c>
-      <c r="D78" s="18" t="inlineStr"/>
-    </row>
-    <row r="79">
-      <c r="B79" s="24" t="inlineStr">
-        <is>
-          <t>#83</t>
-        </is>
-      </c>
-      <c r="C79" s="15" t="n">
-        <v>46299</v>
-      </c>
-      <c r="D79" s="18" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="B80" s="24" t="inlineStr">
         <is>
-          <t>#84</t>
+          <t>#81</t>
         </is>
       </c>
       <c r="C80" s="15" t="n">
-        <v>46302</v>
-      </c>
-      <c r="D80" s="18" t="inlineStr"/>
+        <v>46293</v>
+      </c>
+      <c r="D80" s="18" t="inlineStr">
+        <is>
+          <t>9월 마지막 Batch (간격 기준점)</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="B81" s="24" t="inlineStr">
         <is>
-          <t>#85</t>
+          <t>#82</t>
         </is>
       </c>
       <c r="C81" s="15" t="n">
-        <v>46305</v>
+        <v>46296</v>
       </c>
       <c r="D81" s="18" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="B82" s="24" t="inlineStr">
         <is>
-          <t>#86</t>
+          <t>#83</t>
         </is>
       </c>
       <c r="C82" s="15" t="n">
-        <v>46307</v>
+        <v>46299</v>
       </c>
       <c r="D82" s="18" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="B83" s="24" t="inlineStr">
         <is>
-          <t>#87</t>
+          <t>#84</t>
         </is>
       </c>
       <c r="C83" s="15" t="n">
-        <v>46310</v>
+        <v>46302</v>
       </c>
       <c r="D83" s="18" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="B84" s="24" t="inlineStr">
         <is>
-          <t>#88</t>
+          <t>#85</t>
         </is>
       </c>
       <c r="C84" s="15" t="n">
-        <v>46313</v>
+        <v>46305</v>
       </c>
       <c r="D84" s="18" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="B85" s="24" t="inlineStr">
         <is>
-          <t>#89</t>
+          <t>#86</t>
         </is>
       </c>
       <c r="C85" s="15" t="n">
-        <v>46315</v>
+        <v>46307</v>
       </c>
       <c r="D85" s="18" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="B86" s="24" t="inlineStr">
         <is>
-          <t>#90</t>
+          <t>#87</t>
         </is>
       </c>
       <c r="C86" s="15" t="n">
-        <v>46318</v>
+        <v>46310</v>
       </c>
       <c r="D86" s="18" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="B87" s="24" t="inlineStr">
         <is>
-          <t>#91</t>
+          <t>#88</t>
         </is>
       </c>
       <c r="C87" s="15" t="n">
-        <v>46321</v>
+        <v>46313</v>
       </c>
       <c r="D87" s="18" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="B88" s="24" t="inlineStr">
         <is>
+          <t>#89</t>
+        </is>
+      </c>
+      <c r="C88" s="15" t="n">
+        <v>46315</v>
+      </c>
+      <c r="D88" s="18" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="B89" s="24" t="inlineStr">
+        <is>
+          <t>#90</t>
+        </is>
+      </c>
+      <c r="C89" s="15" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D89" s="18" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="B90" s="24" t="inlineStr">
+        <is>
+          <t>#91</t>
+        </is>
+      </c>
+      <c r="C90" s="15" t="n">
+        <v>46321</v>
+      </c>
+      <c r="D90" s="18" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="B91" s="24" t="inlineStr">
+        <is>
           <t>#92</t>
         </is>
       </c>
-      <c r="C88" s="15" t="n">
+      <c r="C91" s="15" t="n">
         <v>46324</v>
       </c>
-      <c r="D88" s="18" t="inlineStr"/>
-    </row>
-    <row r="89">
-      <c r="B89" s="18" t="inlineStr">
+      <c r="D91" s="18" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="B92" s="18" t="inlineStr">
         <is>
           <t>10월 완료 #82~#92 = 11 Batch · 행을 추가하면 03_Batch주기 계산 범위도 같이 조정</t>
         </is>
@@ -2333,17 +2393,17 @@
       </c>
       <c r="C16" s="50" t="inlineStr">
         <is>
-          <t>9병 18 h 작업, 근무시간 반영 시 약 2일 · 개선 방향 1~1.5일 · 18 h → 9 h 방안 검토</t>
+          <t>9병 18 h 작업 · 충진은 보통 상근조(08:00~17:00, 점심 12~13시 제외 = 8 h/일)만 진행 → 약 2일 · 개선 방향 1~1.5일 · 18 h → 9 h 방안 검토</t>
         </is>
       </c>
       <c r="D16" s="50" t="inlineStr">
         <is>
-          <t>2 h/병 · 18 h 유지 (개선은 미반영)</t>
+          <t>2 h/병 · 18 h 유지 · 상근조 8 h/일 기준 약 2일 (개선은 미반영)</t>
         </is>
       </c>
       <c r="E16" s="50" t="inlineStr">
         <is>
-          <t>교대·연장근무 · 충진 인원</t>
+          <t>18 h ÷ 8 h = 2.25일 → 9병째가 3일차로 넘어가는지 · 연장근무·교대 충진 가능 여부 · 인원</t>
         </is>
       </c>
     </row>
@@ -3904,7 +3964,7 @@
     <row r="22">
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>5 Gal 9병 충진 경과 (근무시간 반영)</t>
+          <t>5 Gal 9병 충진 경과 (상근조 8 h/일)</t>
         </is>
       </c>
       <c r="C22" s="28">
@@ -3918,7 +3978,7 @@
       </c>
       <c r="E22" s="18" t="inlineStr">
         <is>
-          <t>현장 설명 약 2일 · 교대·연장근무 조건 확인</t>
+          <t>상근조 08~17시 · 점심 1 h 제외 → 현장 설명 약 2일</t>
         </is>
       </c>
     </row>
@@ -4041,11 +4101,11 @@
     </row>
     <row r="6">
       <c r="B6" s="5" t="str">
-        <f>'01_입력'!B77</f>
+        <f>'01_입력'!B80</f>
         <v>#81</v>
       </c>
       <c r="C6" s="29">
-        <f>'01_입력'!C77</f>
+        <f>'01_입력'!C80</f>
         <v>46293.0</v>
       </c>
       <c r="D6" s="5" t="str">
@@ -4065,11 +4125,11 @@
     </row>
     <row r="7">
       <c r="B7" s="5" t="str">
-        <f>'01_입력'!B78</f>
+        <f>'01_입력'!B81</f>
         <v>#82</v>
       </c>
       <c r="C7" s="29">
-        <f>'01_입력'!C78</f>
+        <f>'01_입력'!C81</f>
         <v>46296.0</v>
       </c>
       <c r="D7" s="5" t="str">
@@ -4095,11 +4155,11 @@
     </row>
     <row r="8">
       <c r="B8" s="5" t="str">
-        <f>'01_입력'!B79</f>
+        <f>'01_입력'!B82</f>
         <v>#83</v>
       </c>
       <c r="C8" s="29">
-        <f>'01_입력'!C79</f>
+        <f>'01_입력'!C82</f>
         <v>46299.0</v>
       </c>
       <c r="D8" s="5" t="str">
@@ -4125,11 +4185,11 @@
     </row>
     <row r="9">
       <c r="B9" s="5" t="str">
-        <f>'01_입력'!B80</f>
+        <f>'01_입력'!B83</f>
         <v>#84</v>
       </c>
       <c r="C9" s="29">
-        <f>'01_입력'!C80</f>
+        <f>'01_입력'!C83</f>
         <v>46302.0</v>
       </c>
       <c r="D9" s="5" t="str">
@@ -4155,11 +4215,11 @@
     </row>
     <row r="10">
       <c r="B10" s="5" t="str">
-        <f>'01_입력'!B81</f>
+        <f>'01_입력'!B84</f>
         <v>#85</v>
       </c>
       <c r="C10" s="29">
-        <f>'01_입력'!C81</f>
+        <f>'01_입력'!C84</f>
         <v>46305.0</v>
       </c>
       <c r="D10" s="5" t="str">
@@ -4185,11 +4245,11 @@
     </row>
     <row r="11">
       <c r="B11" s="5" t="str">
-        <f>'01_입력'!B82</f>
+        <f>'01_입력'!B85</f>
         <v>#86</v>
       </c>
       <c r="C11" s="29">
-        <f>'01_입력'!C82</f>
+        <f>'01_입력'!C85</f>
         <v>46307.0</v>
       </c>
       <c r="D11" s="5" t="str">
@@ -4215,11 +4275,11 @@
     </row>
     <row r="12">
       <c r="B12" s="5" t="str">
-        <f>'01_입력'!B83</f>
+        <f>'01_입력'!B86</f>
         <v>#87</v>
       </c>
       <c r="C12" s="29">
-        <f>'01_입력'!C83</f>
+        <f>'01_입력'!C86</f>
         <v>46310.0</v>
       </c>
       <c r="D12" s="5" t="str">
@@ -4245,11 +4305,11 @@
     </row>
     <row r="13">
       <c r="B13" s="5" t="str">
-        <f>'01_입력'!B84</f>
+        <f>'01_입력'!B87</f>
         <v>#88</v>
       </c>
       <c r="C13" s="29">
-        <f>'01_입력'!C84</f>
+        <f>'01_입력'!C87</f>
         <v>46313.0</v>
       </c>
       <c r="D13" s="5" t="str">
@@ -4275,11 +4335,11 @@
     </row>
     <row r="14">
       <c r="B14" s="5" t="str">
-        <f>'01_입력'!B85</f>
+        <f>'01_입력'!B88</f>
         <v>#89</v>
       </c>
       <c r="C14" s="29">
-        <f>'01_입력'!C85</f>
+        <f>'01_입력'!C88</f>
         <v>46315.0</v>
       </c>
       <c r="D14" s="5" t="str">
@@ -4305,11 +4365,11 @@
     </row>
     <row r="15">
       <c r="B15" s="5" t="str">
-        <f>'01_입력'!B86</f>
+        <f>'01_입력'!B89</f>
         <v>#90</v>
       </c>
       <c r="C15" s="29">
-        <f>'01_입력'!C86</f>
+        <f>'01_입력'!C89</f>
         <v>46318.0</v>
       </c>
       <c r="D15" s="5" t="str">
@@ -4335,11 +4395,11 @@
     </row>
     <row r="16">
       <c r="B16" s="5" t="str">
-        <f>'01_입력'!B87</f>
+        <f>'01_입력'!B90</f>
         <v>#91</v>
       </c>
       <c r="C16" s="29">
-        <f>'01_입력'!C87</f>
+        <f>'01_입력'!C90</f>
         <v>46321.0</v>
       </c>
       <c r="D16" s="5" t="str">
@@ -4365,11 +4425,11 @@
     </row>
     <row r="17">
       <c r="B17" s="5" t="str">
-        <f>'01_입력'!B88</f>
+        <f>'01_입력'!B91</f>
         <v>#92</v>
       </c>
       <c r="C17" s="29">
-        <f>'01_입력'!C88</f>
+        <f>'01_입력'!C91</f>
         <v>46324.0</v>
       </c>
       <c r="D17" s="5" t="str">
@@ -4602,7 +4662,7 @@
     <row r="32">
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>5 Gal 9병 충진 (근무시간)</t>
+          <t>5 Gal 9병 충진 (상근조)</t>
         </is>
       </c>
       <c r="C32" s="17">
@@ -4627,7 +4687,7 @@
       </c>
       <c r="H32" s="12" t="inlineStr">
         <is>
-          <t>1교대 · 현장 설명 약 2일</t>
+          <t>상근조 8 h/일 · 현장 설명 약 2일</t>
         </is>
       </c>
     </row>
@@ -10324,7 +10384,7 @@
     <row r="9">
       <c r="B9" s="10" t="inlineStr">
         <is>
-          <t>글로브 박스 가용 h (1교대)</t>
+          <t>글로브 박스 가용 h (상근조)</t>
         </is>
       </c>
       <c r="C9" s="30">

</xml_diff>